<commit_message>
adicionando tabela para calculo de aderencia
</commit_message>
<xml_diff>
--- a/Artefato 1.xlsx
+++ b/Artefato 1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pucpredu-my.sharepoint.com/personal/ferrarini_isabela_pucpr_edu_br/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rafael Fernandes\Downloads\ChecklistQualidade\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D402C22F-1026-45B1-A121-CE91E111B465}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8054943-FD90-494A-A447-990CDF007192}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4672E65F-BD16-49AF-B984-110D5D3DB6D8}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="42">
   <si>
     <t xml:space="preserve">Resultado </t>
   </si>
@@ -150,13 +150,28 @@
   </si>
   <si>
     <t>Mariana</t>
+  </si>
+  <si>
+    <t>Aderência Por Área</t>
+  </si>
+  <si>
+    <t>Total de Perguntas</t>
+  </si>
+  <si>
+    <t>Sim</t>
+  </si>
+  <si>
+    <t>Não Aplicavél</t>
+  </si>
+  <si>
+    <t>Aderência</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -178,6 +193,29 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -188,7 +226,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.749992370372631"/>
+        <fgColor rgb="FFA6124E"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -246,20 +284,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -271,14 +303,34 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -297,7 +349,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -613,11 +665,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63381509-777B-4F7A-965D-F5E2BE998752}">
-  <dimension ref="B1:I30"/>
+  <dimension ref="B2:I31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="8.88671875" style="6"/>
-    <col min="3" max="3" width="35.77734375" style="4" customWidth="1"/>
+    <col min="1" max="1" width="7.33203125" customWidth="1"/>
+    <col min="2" max="2" width="11.44140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.77734375" style="3" customWidth="1"/>
     <col min="4" max="4" width="19.5546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.5546875" customWidth="1"/>
     <col min="6" max="6" width="13" customWidth="1"/>
@@ -626,107 +679,126 @@
     <col min="9" max="9" width="21.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C1" s="10" t="s">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C2" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="12"/>
-    </row>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C2" s="11" t="s">
+      <c r="D2" s="17"/>
+      <c r="F2" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+    </row>
+    <row r="3" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C3" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C3" s="11" t="s">
+      <c r="F3" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="I3" s="11" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C4" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C4" s="11" t="s">
+      <c r="F4" s="12"/>
+      <c r="G4" s="13"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="13"/>
+    </row>
+    <row r="5" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C5" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C5" s="11"/>
-      <c r="D5" s="1"/>
+      <c r="F5" s="1">
+        <v>0</v>
+      </c>
+      <c r="G5" s="1">
+        <v>0</v>
+      </c>
+      <c r="H5" s="1">
+        <v>0</v>
+      </c>
+      <c r="I5" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="8"/>
+      <c r="D6" s="1"/>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C7" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C7" s="11" t="s">
+    <row r="8" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C8" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="D7" s="1"/>
-      <c r="G7" s="13"/>
-    </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C8" s="11" t="s">
+      <c r="D8" s="1"/>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C9" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="D8" s="1"/>
-    </row>
-    <row r="10" spans="2:9" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="5" t="s">
+      <c r="D9" s="1"/>
+    </row>
+    <row r="11" spans="2:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="10"/>
-      <c r="D10" s="2" t="s">
+      <c r="C11" s="15"/>
+      <c r="D11" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E11" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F11" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G11" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H11" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="I11" s="16" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="2:9" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="B11" s="7">
+    <row r="12" spans="2:9" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="B12" s="5">
         <v>1</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C12" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D11" s="8"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
-    </row>
-    <row r="12" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="B12" s="7">
-        <v>2</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D12" s="8"/>
+      <c r="D12" s="6"/>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
@@ -734,13 +806,13 @@
       <c r="I12" s="1"/>
     </row>
     <row r="13" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="B13" s="7">
-        <v>3</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="D13" s="8"/>
+      <c r="B13" s="5">
+        <v>2</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="6"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
@@ -748,13 +820,13 @@
       <c r="I13" s="1"/>
     </row>
     <row r="14" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="B14" s="7">
-        <v>4</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="D14" s="8"/>
+      <c r="B14" s="5">
+        <v>3</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" s="6"/>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
@@ -762,41 +834,41 @@
       <c r="I14" s="1"/>
     </row>
     <row r="15" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="B15" s="7">
-        <v>5</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="D15" s="8"/>
+      <c r="B15" s="5">
+        <v>4</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" s="6"/>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
     </row>
-    <row r="16" spans="2:9" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="B16" s="7">
-        <v>6</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D16" s="8"/>
+    <row r="16" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B16" s="5">
+        <v>5</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" s="6"/>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
     </row>
-    <row r="17" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="B17" s="7">
-        <v>7</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="D17" s="8"/>
+    <row r="17" spans="2:9" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="B17" s="5">
+        <v>6</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="6"/>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
@@ -804,13 +876,13 @@
       <c r="I17" s="1"/>
     </row>
     <row r="18" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="B18" s="7">
-        <v>8</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D18" s="8"/>
+      <c r="B18" s="5">
+        <v>7</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" s="6"/>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
@@ -818,27 +890,27 @@
       <c r="I18" s="1"/>
     </row>
     <row r="19" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="B19" s="7">
-        <v>9</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="D19" s="8"/>
+      <c r="B19" s="5">
+        <v>8</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" s="6"/>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
     </row>
-    <row r="20" spans="2:9" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="B20" s="7">
-        <v>10</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="D20" s="8"/>
+    <row r="20" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B20" s="5">
+        <v>9</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" s="6"/>
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
@@ -846,55 +918,55 @@
       <c r="I20" s="1"/>
     </row>
     <row r="21" spans="2:9" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="B21" s="7">
-        <v>11</v>
-      </c>
-      <c r="C21" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D21" s="8"/>
+      <c r="B21" s="5">
+        <v>10</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D21" s="6"/>
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
     </row>
-    <row r="22" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="B22" s="7">
-        <v>12</v>
-      </c>
-      <c r="C22" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="D22" s="8"/>
+    <row r="22" spans="2:9" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="B22" s="5">
+        <v>11</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D22" s="6"/>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
     </row>
-    <row r="23" spans="2:9" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="B23" s="7">
-        <v>13</v>
-      </c>
-      <c r="C23" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D23" s="8"/>
+    <row r="23" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B23" s="5">
+        <v>12</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D23" s="6"/>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
     </row>
-    <row r="24" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="B24" s="7">
-        <v>14</v>
-      </c>
-      <c r="C24" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="D24" s="8"/>
+    <row r="24" spans="2:9" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="B24" s="5">
+        <v>13</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D24" s="6"/>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
@@ -902,27 +974,27 @@
       <c r="I24" s="1"/>
     </row>
     <row r="25" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="B25" s="7">
-        <v>15</v>
-      </c>
-      <c r="C25" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="D25" s="8"/>
+      <c r="B25" s="5">
+        <v>14</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D25" s="6"/>
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
     </row>
-    <row r="26" spans="2:9" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="B26" s="7">
-        <v>16</v>
-      </c>
-      <c r="C26" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="D26" s="8"/>
+    <row r="26" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B26" s="5">
+        <v>15</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D26" s="6"/>
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
@@ -930,13 +1002,13 @@
       <c r="I26" s="1"/>
     </row>
     <row r="27" spans="2:9" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="B27" s="7">
-        <v>17</v>
-      </c>
-      <c r="C27" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="D27" s="8"/>
+      <c r="B27" s="5">
+        <v>16</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D27" s="6"/>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
@@ -944,54 +1016,92 @@
       <c r="I27" s="1"/>
     </row>
     <row r="28" spans="2:9" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="B28" s="7">
-        <v>18</v>
-      </c>
-      <c r="C28" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D28" s="8"/>
+      <c r="B28" s="5">
+        <v>17</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D28" s="6"/>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
     </row>
-    <row r="29" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="B29" s="7">
-        <v>19</v>
-      </c>
-      <c r="C29" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="D29" s="8"/>
+    <row r="29" spans="2:9" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="B29" s="5">
+        <v>18</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D29" s="6"/>
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
     </row>
-    <row r="30" spans="2:9" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="B30" s="7">
-        <v>20</v>
-      </c>
-      <c r="C30" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="D30" s="8"/>
+    <row r="30" spans="2:9" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B30" s="5">
+        <v>19</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D30" s="6"/>
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
       <c r="I30" s="1"/>
     </row>
+    <row r="31" spans="2:9" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="B31" s="5">
+        <v>20</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D31" s="6"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+      <c r="H31" s="1"/>
+      <c r="I31" s="1"/>
+    </row>
   </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="F2:I2"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="H3:H4"/>
+    <mergeCell ref="I3:I4"/>
+  </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="aed73f09-bf5d-4147-a3d9-eca4840d3416" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101007CCF20922A0DE34DA3357EDA40AE3850" ma:contentTypeVersion="5" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="df2c289d3a08b18055ba2ef47a57998b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="aed73f09-bf5d-4147-a3d9-eca4840d3416" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="91dac5f1c2bd6141b57005fd2a16424c" ns3:_="">
     <xsd:import namespace="aed73f09-bf5d-4147-a3d9-eca4840d3416"/>
@@ -1141,24 +1251,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD41F362-A534-43BD-873B-83E80A9078F7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="aed73f09-bf5d-4147-a3d9-eca4840d3416"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="aed73f09-bf5d-4147-a3d9-eca4840d3416" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{901F3B13-F474-42C6-B910-1EF2E5DFC5CC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FC09F85-4182-458C-9936-A4A27B890011}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1174,28 +1291,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{901F3B13-F474-42C6-B910-1EF2E5DFC5CC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD41F362-A534-43BD-873B-83E80A9078F7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="aed73f09-bf5d-4147-a3d9-eca4840d3416"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>